<commit_message>
Add VZT 2.1 photos with draft captions
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DkBvnLE3negxmtmFidQ4SP
</commit_message>
<xml_diff>
--- a/vystupy/Fotodokumentace_VZT_prehled.xlsx
+++ b/vystupy/Fotodokumentace_VZT_prehled.xlsx
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="45">
   <si>
     <t xml:space="preserve">Přehled fotodokumentace úprav VZT – Mondelez Werk 2</t>
   </si>
@@ -137,6 +137,21 @@
   </si>
   <si>
     <t xml:space="preserve">Fotodokumentace provedených úprav – VZT 2.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rozbočovací krabice – svorkovnice N, PE, L1, L2, L3 s označenými vodiči, přívod v ohebné chráničce.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rozvaděč jednotky Systemair – řídicí jednotka, jističe F1–F3, zdroj 24 V (T24), svorkovnice X1.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Uzavřená rozbočovací krabice na boku jednotky, kabel vedený ohebnou chráničkou.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pohled na střechu – izolované potrubí na podpůrné konstrukci, jednotka s krytem.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Detail řídicí jednotky Systemair – komunikační svorky, síťový kabel, vstupy a výstupy.</t>
   </si>
   <si>
     <t xml:space="preserve">Fotodokumentace provedených úprav – VZT 2.2</t>
@@ -469,13 +484,203 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
+      <xdr:colOff>2370960</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>2370960</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="0" name="Image 1" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1236240" y="828720"/>
+          <a:ext cx="2332800" cy="2332800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>38160</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>38160</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>2370960</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>2370960</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="Image 2" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId2"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1236240" y="3238560"/>
+          <a:ext cx="2332800" cy="2332800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>38160</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>38160</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>2370960</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>2370960</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Image 3" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId3"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1236240" y="5648400"/>
+          <a:ext cx="2332800" cy="2332800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>38160</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>38160</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>2370960</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>2370960</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Image 4" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId4"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1236240" y="8058240"/>
+          <a:ext cx="2332800" cy="2332800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>38160</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>38160</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>2370960</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>2370960</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Image 5" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId5"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1236240" y="10468080"/>
+          <a:ext cx="2332800" cy="2332800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>38160</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>38160</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
       <xdr:colOff>2371320</xdr:colOff>
       <xdr:row>4</xdr:row>
       <xdr:rowOff>2371320</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="Image 1" descr="Picture"/>
+        <xdr:cNvPr id="5" name="Image 1" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -512,7 +717,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="Image 2" descr="Picture"/>
+        <xdr:cNvPr id="6" name="Image 2" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -549,7 +754,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Image 3" descr="Picture"/>
+        <xdr:cNvPr id="7" name="Image 3" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -586,7 +791,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Image 4" descr="Picture"/>
+        <xdr:cNvPr id="8" name="Image 4" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -623,7 +828,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Image 5" descr="Picture"/>
+        <xdr:cNvPr id="9" name="Image 5" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -894,7 +1099,7 @@
       </c>
       <c r="B7" s="6" t="n">
         <f aca="false">COUNTA('VZT 2.1'!D5:D24)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="C7" s="7" t="str">
         <f aca="false">IF(COUNT('VZT 2.1'!B5:B24)=0,"",MAX('VZT 2.1'!B5:B24))</f>
@@ -1020,7 +1225,7 @@
       </c>
       <c r="B16" s="9" t="n">
         <f aca="false">SUM(B5:B15)</f>
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C16" s="10"/>
       <c r="D16" s="10"/>
@@ -1064,7 +1269,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1272,7 +1477,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1480,7 +1685,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2143,7 +2348,9 @@
       </c>
       <c r="B5" s="13"/>
       <c r="C5" s="14"/>
-      <c r="D5" s="15"/>
+      <c r="D5" s="15" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="189.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="12" t="n">
@@ -2151,7 +2358,9 @@
       </c>
       <c r="B6" s="13"/>
       <c r="C6" s="14"/>
-      <c r="D6" s="15"/>
+      <c r="D6" s="15" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="189.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="12" t="n">
@@ -2159,7 +2368,9 @@
       </c>
       <c r="B7" s="13"/>
       <c r="C7" s="14"/>
-      <c r="D7" s="15"/>
+      <c r="D7" s="15" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="189.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="12" t="n">
@@ -2167,7 +2378,9 @@
       </c>
       <c r="B8" s="13"/>
       <c r="C8" s="14"/>
-      <c r="D8" s="15"/>
+      <c r="D8" s="15" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="189.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="12" t="n">
@@ -2175,7 +2388,9 @@
       </c>
       <c r="B9" s="13"/>
       <c r="C9" s="14"/>
-      <c r="D9" s="15"/>
+      <c r="D9" s="15" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="189.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="12" t="n">
@@ -2305,6 +2520,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2323,7 +2539,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2531,7 +2747,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2739,7 +2955,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2947,7 +3163,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3156,7 +3372,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3169,7 +3385,7 @@
         <v>20</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="C4" s="11" t="s">
         <v>21</v>

</xml_diff>

<commit_message>
Add VZT 3.1 photos with draft captions
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DkBvnLE3negxmtmFidQ4SP
</commit_message>
<xml_diff>
--- a/vystupy/Fotodokumentace_VZT_prehled.xlsx
+++ b/vystupy/Fotodokumentace_VZT_prehled.xlsx
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="50">
   <si>
     <t xml:space="preserve">Přehled fotodokumentace úprav VZT – Mondelez Werk 2</t>
   </si>
@@ -158,6 +158,21 @@
   </si>
   <si>
     <t xml:space="preserve">Fotodokumentace provedených úprav – VZT 3.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Čelní panel jednotky Daikin – kontrolky GENERAL ALARM (červená) a SYSTEM (zelená), pod ním kabelové průchodky; průhledné okno zamlžené.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Přívod napájení – jistič ABB Tmax XT1 (In = 32 A), proudový chránič F202 25 A / 30 mA, přípojka PE, štítek EXTERNAL POWER SUPPLY.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Celkový pohled na jednotku Daikin na střeše – panel s nouzovým STOP, izolované potrubí na ocelové konstrukci, zábradlí.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Detail podlahy jednotky – potrubí v prostupu s třmenem, závitové tyče, stopy rzi a nečistot na plechu.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pohled na jednotku a okolí – volně položené kabely na střeše, ocelová konstrukce, střešní ventilátor.</t>
   </si>
   <si>
     <t xml:space="preserve">Fotodokumentace provedených úprav – VZT 3.2</t>
@@ -484,13 +499,203 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
+      <xdr:colOff>2370600</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>2370600</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="0" name="Image 1" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1236240" y="828720"/>
+          <a:ext cx="2332440" cy="2332440"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>38160</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>38160</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>2370600</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>2370600</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="Image 2" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId2"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1236240" y="3238560"/>
+          <a:ext cx="2332440" cy="2332440"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>38160</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>38160</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>2370600</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>2370600</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Image 3" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId3"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1236240" y="5648400"/>
+          <a:ext cx="2332440" cy="2332440"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>38160</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>38160</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>2370600</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>2370600</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Image 4" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId4"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1236240" y="8058240"/>
+          <a:ext cx="2332440" cy="2332440"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>38160</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>38160</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>2370600</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>2370600</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Image 5" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId5"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1236240" y="10468080"/>
+          <a:ext cx="2332440" cy="2332440"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>38160</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>38160</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
       <xdr:colOff>2370960</xdr:colOff>
       <xdr:row>4</xdr:row>
       <xdr:rowOff>2370960</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="Image 1" descr="Picture"/>
+        <xdr:cNvPr id="5" name="Image 1" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -527,7 +732,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="Image 2" descr="Picture"/>
+        <xdr:cNvPr id="6" name="Image 2" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -564,7 +769,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Image 3" descr="Picture"/>
+        <xdr:cNvPr id="7" name="Image 3" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -601,7 +806,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Image 4" descr="Picture"/>
+        <xdr:cNvPr id="8" name="Image 4" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -638,7 +843,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Image 5" descr="Picture"/>
+        <xdr:cNvPr id="9" name="Image 5" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -663,7 +868,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -674,13 +879,13 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>2371320</xdr:colOff>
+      <xdr:colOff>1085400</xdr:colOff>
       <xdr:row>4</xdr:row>
       <xdr:rowOff>2371320</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="Image 1" descr="Picture"/>
+        <xdr:cNvPr id="10" name="Image 1" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -690,7 +895,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="1236240" y="828720"/>
-          <a:ext cx="2333160" cy="2333160"/>
+          <a:ext cx="1047240" cy="2333160"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -711,13 +916,13 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>2371320</xdr:colOff>
+      <xdr:colOff>1085400</xdr:colOff>
       <xdr:row>5</xdr:row>
       <xdr:rowOff>2371320</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="6" name="Image 2" descr="Picture"/>
+        <xdr:cNvPr id="11" name="Image 2" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -727,7 +932,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="1236240" y="3238560"/>
-          <a:ext cx="2333160" cy="2333160"/>
+          <a:ext cx="1047240" cy="2333160"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -750,11 +955,11 @@
       <xdr:col>2</xdr:col>
       <xdr:colOff>2371320</xdr:colOff>
       <xdr:row>6</xdr:row>
-      <xdr:rowOff>2371320</xdr:rowOff>
+      <xdr:rowOff>1085400</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="7" name="Image 3" descr="Picture"/>
+        <xdr:cNvPr id="12" name="Image 3" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -764,7 +969,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="1236240" y="5648400"/>
-          <a:ext cx="2333160" cy="2333160"/>
+          <a:ext cx="2333160" cy="1047240"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -785,13 +990,13 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>2371320</xdr:colOff>
+      <xdr:colOff>1085400</xdr:colOff>
       <xdr:row>7</xdr:row>
       <xdr:rowOff>2371320</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="8" name="Image 4" descr="Picture"/>
+        <xdr:cNvPr id="13" name="Image 4" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -801,7 +1006,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="1236240" y="8058240"/>
-          <a:ext cx="2333160" cy="2333160"/>
+          <a:ext cx="1047240" cy="2333160"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -828,7 +1033,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="9" name="Image 5" descr="Picture"/>
+        <xdr:cNvPr id="14" name="Image 5" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -1127,7 +1332,7 @@
       </c>
       <c r="B9" s="6" t="n">
         <f aca="false">COUNTA('VZT 3.1'!D5:D24)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="C9" s="7" t="str">
         <f aca="false">IF(COUNT('VZT 3.1'!B5:B24)=0,"",MAX('VZT 3.1'!B5:B24))</f>
@@ -1225,7 +1430,7 @@
       </c>
       <c r="B16" s="9" t="n">
         <f aca="false">SUM(B5:B15)</f>
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="C16" s="10"/>
       <c r="D16" s="10"/>
@@ -1269,7 +1474,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1477,7 +1682,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1685,7 +1890,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2775,7 +2980,9 @@
       </c>
       <c r="B5" s="13"/>
       <c r="C5" s="14"/>
-      <c r="D5" s="15"/>
+      <c r="D5" s="15" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="189.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="12" t="n">
@@ -2783,7 +2990,9 @@
       </c>
       <c r="B6" s="13"/>
       <c r="C6" s="14"/>
-      <c r="D6" s="15"/>
+      <c r="D6" s="15" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="189.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="12" t="n">
@@ -2791,7 +3000,9 @@
       </c>
       <c r="B7" s="13"/>
       <c r="C7" s="14"/>
-      <c r="D7" s="15"/>
+      <c r="D7" s="15" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="189.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="12" t="n">
@@ -2799,7 +3010,9 @@
       </c>
       <c r="B8" s="13"/>
       <c r="C8" s="14"/>
-      <c r="D8" s="15"/>
+      <c r="D8" s="15" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="189.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="12" t="n">
@@ -2807,7 +3020,9 @@
       </c>
       <c r="B9" s="13"/>
       <c r="C9" s="14"/>
-      <c r="D9" s="15"/>
+      <c r="D9" s="15" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="189.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="12" t="n">
@@ -2937,6 +3152,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2955,7 +3171,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3163,7 +3379,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3372,7 +3588,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3385,7 +3601,7 @@
         <v>20</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="C4" s="11" t="s">
         <v>21</v>

</xml_diff>

<commit_message>
Add VZT 4.1 photos with draft captions
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DkBvnLE3negxmtmFidQ4SP
</commit_message>
<xml_diff>
--- a/vystupy/Fotodokumentace_VZT_prehled.xlsx
+++ b/vystupy/Fotodokumentace_VZT_prehled.xlsx
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="55">
   <si>
     <t xml:space="preserve">Přehled fotodokumentace úprav VZT – Mondelez Werk 2</t>
   </si>
@@ -179,6 +179,21 @@
   </si>
   <si>
     <t xml:space="preserve">Fotodokumentace provedených úprav – VZT 4.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Detail řídicí jednotky MicroTech 4 (MT3105) – komunikační kabel s konektorem RJ45, označený šedý kabel, svorkovnice 101–126.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Otevřený rozvaděč jednotky – hlavní vypínač ABB QS1, pojistky FU1–FU7, regulátor MicroTech 4, svorkovnice.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vodní větev v jednotce – lisované pozinkované potrubí, třícestný ventil s pohonem, odvzdušňovací ventil, označení spojů.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pohled podél výměníku – manometry, ventily, kabeláž vedená po stropě jednotky a řídicí modul Daikin.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ventilátorová sekce – radiální ventilátor, kabely stažené páskami; v sekci odložené krabice s příslušenstvím Daikin, filtry a dokumentace.</t>
   </si>
   <si>
     <t xml:space="preserve">Fotodokumentace provedených úprav – VZT 4.2 a_b_c_d</t>
@@ -499,13 +514,203 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
+      <xdr:colOff>2370240</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>2370240</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="0" name="Image 1" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1236240" y="828720"/>
+          <a:ext cx="2332080" cy="2332080"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>38160</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>38160</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>2370240</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>2370240</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="Image 2" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId2"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1236240" y="3238560"/>
+          <a:ext cx="2332080" cy="2332080"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>38160</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>38160</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>2370240</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>2370240</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Image 3" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId3"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1236240" y="5648400"/>
+          <a:ext cx="2332080" cy="2332080"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>38160</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>38160</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>2370240</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>2370240</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Image 4" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId4"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1236240" y="8058240"/>
+          <a:ext cx="2332080" cy="2332080"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>38160</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>38160</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>2370240</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>2370240</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Image 5" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId5"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1236240" y="10468080"/>
+          <a:ext cx="2332080" cy="2332080"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>38160</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>38160</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
       <xdr:colOff>2370600</xdr:colOff>
       <xdr:row>4</xdr:row>
       <xdr:rowOff>2370600</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="Image 1" descr="Picture"/>
+        <xdr:cNvPr id="5" name="Image 1" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -542,7 +747,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="Image 2" descr="Picture"/>
+        <xdr:cNvPr id="6" name="Image 2" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -579,7 +784,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Image 3" descr="Picture"/>
+        <xdr:cNvPr id="7" name="Image 3" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -616,7 +821,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Image 4" descr="Picture"/>
+        <xdr:cNvPr id="8" name="Image 4" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -653,7 +858,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Image 5" descr="Picture"/>
+        <xdr:cNvPr id="9" name="Image 5" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -678,7 +883,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -689,13 +894,13 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>2370960</xdr:colOff>
+      <xdr:colOff>1085040</xdr:colOff>
       <xdr:row>4</xdr:row>
       <xdr:rowOff>2370960</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="Image 1" descr="Picture"/>
+        <xdr:cNvPr id="10" name="Image 1" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -705,7 +910,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="1236240" y="828720"/>
-          <a:ext cx="2332800" cy="2332800"/>
+          <a:ext cx="1046880" cy="2332800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -726,13 +931,13 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>2370960</xdr:colOff>
+      <xdr:colOff>1085040</xdr:colOff>
       <xdr:row>5</xdr:row>
       <xdr:rowOff>2370960</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="6" name="Image 2" descr="Picture"/>
+        <xdr:cNvPr id="11" name="Image 2" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -742,7 +947,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="1236240" y="3238560"/>
-          <a:ext cx="2332800" cy="2332800"/>
+          <a:ext cx="1046880" cy="2332800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -765,11 +970,11 @@
       <xdr:col>2</xdr:col>
       <xdr:colOff>2370960</xdr:colOff>
       <xdr:row>6</xdr:row>
-      <xdr:rowOff>2370960</xdr:rowOff>
+      <xdr:rowOff>1085040</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="7" name="Image 3" descr="Picture"/>
+        <xdr:cNvPr id="12" name="Image 3" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -779,7 +984,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="1236240" y="5648400"/>
-          <a:ext cx="2332800" cy="2332800"/>
+          <a:ext cx="2332800" cy="1046880"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -800,13 +1005,13 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>2370960</xdr:colOff>
+      <xdr:colOff>1085040</xdr:colOff>
       <xdr:row>7</xdr:row>
       <xdr:rowOff>2370960</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="8" name="Image 4" descr="Picture"/>
+        <xdr:cNvPr id="13" name="Image 4" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -816,7 +1021,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="1236240" y="8058240"/>
-          <a:ext cx="2332800" cy="2332800"/>
+          <a:ext cx="1046880" cy="2332800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -843,7 +1048,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="9" name="Image 5" descr="Picture"/>
+        <xdr:cNvPr id="14" name="Image 5" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -868,7 +1073,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -879,13 +1084,13 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>1085400</xdr:colOff>
+      <xdr:colOff>2371320</xdr:colOff>
       <xdr:row>4</xdr:row>
       <xdr:rowOff>2371320</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="10" name="Image 1" descr="Picture"/>
+        <xdr:cNvPr id="15" name="Image 1" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -895,7 +1100,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="1236240" y="828720"/>
-          <a:ext cx="1047240" cy="2333160"/>
+          <a:ext cx="2333160" cy="2333160"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -916,13 +1121,13 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>1085400</xdr:colOff>
+      <xdr:colOff>2371320</xdr:colOff>
       <xdr:row>5</xdr:row>
       <xdr:rowOff>2371320</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="11" name="Image 2" descr="Picture"/>
+        <xdr:cNvPr id="16" name="Image 2" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -932,7 +1137,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="1236240" y="3238560"/>
-          <a:ext cx="1047240" cy="2333160"/>
+          <a:ext cx="2333160" cy="2333160"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -955,11 +1160,11 @@
       <xdr:col>2</xdr:col>
       <xdr:colOff>2371320</xdr:colOff>
       <xdr:row>6</xdr:row>
-      <xdr:rowOff>1085400</xdr:rowOff>
+      <xdr:rowOff>2371320</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="12" name="Image 3" descr="Picture"/>
+        <xdr:cNvPr id="17" name="Image 3" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -969,7 +1174,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="1236240" y="5648400"/>
-          <a:ext cx="2333160" cy="1047240"/>
+          <a:ext cx="2333160" cy="2333160"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -990,13 +1195,13 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>1085400</xdr:colOff>
+      <xdr:colOff>2371320</xdr:colOff>
       <xdr:row>7</xdr:row>
       <xdr:rowOff>2371320</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="13" name="Image 4" descr="Picture"/>
+        <xdr:cNvPr id="18" name="Image 4" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -1006,7 +1211,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="1236240" y="8058240"/>
-          <a:ext cx="1047240" cy="2333160"/>
+          <a:ext cx="2333160" cy="2333160"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1033,7 +1238,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="14" name="Image 5" descr="Picture"/>
+        <xdr:cNvPr id="19" name="Image 5" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -1360,7 +1565,7 @@
       </c>
       <c r="B11" s="6" t="n">
         <f aca="false">COUNTA('VZT 4.1'!D5:D24)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="C11" s="7" t="str">
         <f aca="false">IF(COUNT('VZT 4.1'!B5:B24)=0,"",MAX('VZT 4.1'!B5:B24))</f>
@@ -1430,7 +1635,7 @@
       </c>
       <c r="B16" s="9" t="n">
         <f aca="false">SUM(B5:B15)</f>
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="C16" s="10"/>
       <c r="D16" s="10"/>
@@ -1474,7 +1679,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1682,7 +1887,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1890,7 +2095,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3407,7 +3612,9 @@
       </c>
       <c r="B5" s="13"/>
       <c r="C5" s="14"/>
-      <c r="D5" s="15"/>
+      <c r="D5" s="15" t="s">
+        <v>45</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="189.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="12" t="n">
@@ -3415,7 +3622,9 @@
       </c>
       <c r="B6" s="13"/>
       <c r="C6" s="14"/>
-      <c r="D6" s="15"/>
+      <c r="D6" s="15" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="189.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="12" t="n">
@@ -3423,7 +3632,9 @@
       </c>
       <c r="B7" s="13"/>
       <c r="C7" s="14"/>
-      <c r="D7" s="15"/>
+      <c r="D7" s="15" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="189.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="12" t="n">
@@ -3431,7 +3642,9 @@
       </c>
       <c r="B8" s="13"/>
       <c r="C8" s="14"/>
-      <c r="D8" s="15"/>
+      <c r="D8" s="15" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="189.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="12" t="n">
@@ -3439,7 +3652,9 @@
       </c>
       <c r="B9" s="13"/>
       <c r="C9" s="14"/>
-      <c r="D9" s="15"/>
+      <c r="D9" s="15" t="s">
+        <v>49</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="189.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="12" t="n">
@@ -3569,6 +3784,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -3588,7 +3804,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3601,7 +3817,7 @@
         <v>20</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="C4" s="11" t="s">
         <v>21</v>

</xml_diff>

<commit_message>
Add VZT 4.2 a_b_c_d photos with draft captions
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DkBvnLE3negxmtmFidQ4SP
</commit_message>
<xml_diff>
--- a/vystupy/Fotodokumentace_VZT_prehled.xlsx
+++ b/vystupy/Fotodokumentace_VZT_prehled.xlsx
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="57">
   <si>
     <t xml:space="preserve">Přehled fotodokumentace úprav VZT – Mondelez Werk 2</t>
   </si>
@@ -200,6 +200,12 @@
   </si>
   <si>
     <t xml:space="preserve">Část (a/b/c/d)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pohled na jednotku Daikin a dvojici venkovních jednotek VRV IV Loop – ocelová konstrukce, lávka se schody a zábradlím, izolované potrubí chladiva.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dvojice venkovních jednotek Daikin VRV IV Loop na ocelovém rámu vedle lávky k vzduchotechnické jednotce; izolované přípojky chladiva.</t>
   </si>
   <si>
     <t xml:space="preserve">Fotodokumentace provedených úprav – VZT 5.1</t>
@@ -514,13 +520,203 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
+      <xdr:colOff>2369880</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>2369880</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="0" name="Image 1" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1236240" y="828720"/>
+          <a:ext cx="2331720" cy="2331720"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>38160</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>38160</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>2369880</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>2369880</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="Image 2" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId2"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1236240" y="3238560"/>
+          <a:ext cx="2331720" cy="2331720"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>38160</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>38160</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>2369880</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>2369880</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Image 3" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId3"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1236240" y="5648400"/>
+          <a:ext cx="2331720" cy="2331720"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>38160</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>38160</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>2369880</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>2369880</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Image 4" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId4"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1236240" y="8058240"/>
+          <a:ext cx="2331720" cy="2331720"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>38160</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>38160</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>2369880</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>2369880</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Image 5" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId5"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1236240" y="10468080"/>
+          <a:ext cx="2331720" cy="2331720"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>38160</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>38160</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
       <xdr:colOff>2370240</xdr:colOff>
       <xdr:row>4</xdr:row>
       <xdr:rowOff>2370240</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="Image 1" descr="Picture"/>
+        <xdr:cNvPr id="5" name="Image 1" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -557,7 +753,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="Image 2" descr="Picture"/>
+        <xdr:cNvPr id="6" name="Image 2" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -594,7 +790,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Image 3" descr="Picture"/>
+        <xdr:cNvPr id="7" name="Image 3" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -631,7 +827,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Image 4" descr="Picture"/>
+        <xdr:cNvPr id="8" name="Image 4" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -668,7 +864,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Image 5" descr="Picture"/>
+        <xdr:cNvPr id="9" name="Image 5" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -693,7 +889,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -704,13 +900,13 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>2370600</xdr:colOff>
+      <xdr:colOff>1084680</xdr:colOff>
       <xdr:row>4</xdr:row>
       <xdr:rowOff>2370600</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="Image 1" descr="Picture"/>
+        <xdr:cNvPr id="10" name="Image 1" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -720,7 +916,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="1236240" y="828720"/>
-          <a:ext cx="2332440" cy="2332440"/>
+          <a:ext cx="1046520" cy="2332440"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -741,13 +937,13 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>2370600</xdr:colOff>
+      <xdr:colOff>1084680</xdr:colOff>
       <xdr:row>5</xdr:row>
       <xdr:rowOff>2370600</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="6" name="Image 2" descr="Picture"/>
+        <xdr:cNvPr id="11" name="Image 2" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -757,7 +953,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="1236240" y="3238560"/>
-          <a:ext cx="2332440" cy="2332440"/>
+          <a:ext cx="1046520" cy="2332440"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -780,11 +976,11 @@
       <xdr:col>2</xdr:col>
       <xdr:colOff>2370600</xdr:colOff>
       <xdr:row>6</xdr:row>
-      <xdr:rowOff>2370600</xdr:rowOff>
+      <xdr:rowOff>1084680</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="7" name="Image 3" descr="Picture"/>
+        <xdr:cNvPr id="12" name="Image 3" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -794,7 +990,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="1236240" y="5648400"/>
-          <a:ext cx="2332440" cy="2332440"/>
+          <a:ext cx="2332440" cy="1046520"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -815,13 +1011,13 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>2370600</xdr:colOff>
+      <xdr:colOff>1084680</xdr:colOff>
       <xdr:row>7</xdr:row>
       <xdr:rowOff>2370600</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="8" name="Image 4" descr="Picture"/>
+        <xdr:cNvPr id="13" name="Image 4" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -831,7 +1027,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="1236240" y="8058240"/>
-          <a:ext cx="2332440" cy="2332440"/>
+          <a:ext cx="1046520" cy="2332440"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -858,7 +1054,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="9" name="Image 5" descr="Picture"/>
+        <xdr:cNvPr id="14" name="Image 5" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -883,7 +1079,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -894,13 +1090,13 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>1085040</xdr:colOff>
+      <xdr:colOff>2370960</xdr:colOff>
       <xdr:row>4</xdr:row>
       <xdr:rowOff>2370960</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="10" name="Image 1" descr="Picture"/>
+        <xdr:cNvPr id="15" name="Image 1" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -910,7 +1106,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="1236240" y="828720"/>
-          <a:ext cx="1046880" cy="2332800"/>
+          <a:ext cx="2332800" cy="2332800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -931,13 +1127,13 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>1085040</xdr:colOff>
+      <xdr:colOff>2370960</xdr:colOff>
       <xdr:row>5</xdr:row>
       <xdr:rowOff>2370960</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="11" name="Image 2" descr="Picture"/>
+        <xdr:cNvPr id="16" name="Image 2" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -947,7 +1143,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="1236240" y="3238560"/>
-          <a:ext cx="1046880" cy="2332800"/>
+          <a:ext cx="2332800" cy="2332800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -970,11 +1166,11 @@
       <xdr:col>2</xdr:col>
       <xdr:colOff>2370960</xdr:colOff>
       <xdr:row>6</xdr:row>
-      <xdr:rowOff>1085040</xdr:rowOff>
+      <xdr:rowOff>2370960</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="12" name="Image 3" descr="Picture"/>
+        <xdr:cNvPr id="17" name="Image 3" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -984,7 +1180,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="1236240" y="5648400"/>
-          <a:ext cx="2332800" cy="1046880"/>
+          <a:ext cx="2332800" cy="2332800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1005,13 +1201,13 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>1085040</xdr:colOff>
+      <xdr:colOff>2370960</xdr:colOff>
       <xdr:row>7</xdr:row>
       <xdr:rowOff>2370960</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="13" name="Image 4" descr="Picture"/>
+        <xdr:cNvPr id="18" name="Image 4" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -1021,7 +1217,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="1236240" y="8058240"/>
-          <a:ext cx="1046880" cy="2332800"/>
+          <a:ext cx="2332800" cy="2332800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1048,7 +1244,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="14" name="Image 5" descr="Picture"/>
+        <xdr:cNvPr id="19" name="Image 5" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -1073,24 +1269,24 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>2</xdr:col>
+      <xdr:col>3</xdr:col>
       <xdr:colOff>38160</xdr:colOff>
       <xdr:row>4</xdr:row>
       <xdr:rowOff>38160</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>2</xdr:col>
+      <xdr:col>3</xdr:col>
       <xdr:colOff>2371320</xdr:colOff>
       <xdr:row>4</xdr:row>
       <xdr:rowOff>2371320</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="15" name="Image 1" descr="Picture"/>
+        <xdr:cNvPr id="20" name="Image 1" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -1099,7 +1295,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1236240" y="828720"/>
+          <a:off x="2223360" y="828720"/>
           <a:ext cx="2333160" cy="2333160"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1114,20 +1310,20 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>2</xdr:col>
+      <xdr:col>3</xdr:col>
       <xdr:colOff>38160</xdr:colOff>
       <xdr:row>5</xdr:row>
       <xdr:rowOff>38160</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>2</xdr:col>
+      <xdr:col>3</xdr:col>
       <xdr:colOff>2371320</xdr:colOff>
       <xdr:row>5</xdr:row>
       <xdr:rowOff>2371320</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="16" name="Image 2" descr="Picture"/>
+        <xdr:cNvPr id="21" name="Image 2" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -1136,118 +1332,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1236240" y="3238560"/>
-          <a:ext cx="2333160" cy="2333160"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="0">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>38160</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>38160</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>2371320</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>2371320</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="17" name="Image 3" descr="Picture"/>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId3"/>
-        <a:stretch/>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="1236240" y="5648400"/>
-          <a:ext cx="2333160" cy="2333160"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="0">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>38160</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>38160</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>2371320</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>2371320</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="18" name="Image 4" descr="Picture"/>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId4"/>
-        <a:stretch/>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="1236240" y="8058240"/>
-          <a:ext cx="2333160" cy="2333160"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="0">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>38160</xdr:colOff>
-      <xdr:row>8</xdr:row>
-      <xdr:rowOff>38160</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>2371320</xdr:colOff>
-      <xdr:row>8</xdr:row>
-      <xdr:rowOff>2371320</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="19" name="Image 5" descr="Picture"/>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId5"/>
-        <a:stretch/>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="1236240" y="10468080"/>
+          <a:off x="2223360" y="3238560"/>
           <a:ext cx="2333160" cy="2333160"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1579,7 +1664,7 @@
       </c>
       <c r="B12" s="6" t="n">
         <f aca="false">COUNTA('VZT 4.2 a_b_c_d'!E5:E24)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C12" s="7" t="str">
         <f aca="false">IF(COUNT('VZT 4.2 a_b_c_d'!C5:C24)=0,"",MAX('VZT 4.2 a_b_c_d'!C5:C24))</f>
@@ -1635,7 +1720,7 @@
       </c>
       <c r="B16" s="9" t="n">
         <f aca="false">SUM(B5:B15)</f>
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C16" s="10"/>
       <c r="D16" s="10"/>
@@ -1679,7 +1764,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1887,7 +1972,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2095,7 +2180,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3836,7 +3921,9 @@
       <c r="B5" s="16"/>
       <c r="C5" s="13"/>
       <c r="D5" s="14"/>
-      <c r="E5" s="15"/>
+      <c r="E5" s="15" t="s">
+        <v>52</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="189.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="12" t="n">
@@ -3845,7 +3932,9 @@
       <c r="B6" s="16"/>
       <c r="C6" s="13"/>
       <c r="D6" s="14"/>
-      <c r="E6" s="15"/>
+      <c r="E6" s="15" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="189.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="12" t="n">
@@ -4017,5 +4106,6 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add VZT 5.1 photos with draft captions
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DkBvnLE3negxmtmFidQ4SP
</commit_message>
<xml_diff>
--- a/vystupy/Fotodokumentace_VZT_prehled.xlsx
+++ b/vystupy/Fotodokumentace_VZT_prehled.xlsx
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="62">
   <si>
     <t xml:space="preserve">Přehled fotodokumentace úprav VZT – Mondelez Werk 2</t>
   </si>
@@ -209,6 +209,21 @@
   </si>
   <si>
     <t xml:space="preserve">Fotodokumentace provedených úprav – VZT 5.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Čelní panel jednotky Daikin – displej, kontrolky GENERAL ALARM a SYSTEM ON, vypínač, nouzové tlačítko EMERGENCY STOP, kabel v ohebné chráničce.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sekce filtrů – dodané kapsové filtry (DriPak GX, ePM10 60 %) zatím v původních krabicích.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vodní větev v jednotce – teploměry/manometry, třícestný ventil s pohonem, vyvažovací ventil, izolované potrubí.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Detail přípojky výměníku – izolované potrubí, odvzdušňovací ventil, kabeláž a řídicí modul Daikin na stropě sekce.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ventilátorová sekce – dva radiální ventilátory, kabeláž upevněná stahovacími páskami, vypouštěcí kohout na dveřích.</t>
   </si>
   <si>
     <t xml:space="preserve">Fotodokumentace provedených úprav – VZT 10.1</t>
@@ -520,13 +535,203 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
+      <xdr:colOff>2369520</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>2369520</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="0" name="Image 1" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1236240" y="828720"/>
+          <a:ext cx="2331360" cy="2331360"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>38160</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>38160</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>2369520</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>2369520</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="Image 2" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId2"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1236240" y="3238560"/>
+          <a:ext cx="2331360" cy="2331360"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>38160</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>38160</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>2369520</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>2369520</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Image 3" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId3"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1236240" y="5648400"/>
+          <a:ext cx="2331360" cy="2331360"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>38160</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>38160</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>2369520</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>2369520</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Image 4" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId4"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1236240" y="8058240"/>
+          <a:ext cx="2331360" cy="2331360"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>38160</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>38160</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>2369520</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>2369520</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Image 5" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId5"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1236240" y="10468080"/>
+          <a:ext cx="2331360" cy="2331360"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>38160</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>38160</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
       <xdr:colOff>2369880</xdr:colOff>
       <xdr:row>4</xdr:row>
       <xdr:rowOff>2369880</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="Image 1" descr="Picture"/>
+        <xdr:cNvPr id="5" name="Image 1" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -563,7 +768,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="Image 2" descr="Picture"/>
+        <xdr:cNvPr id="6" name="Image 2" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -600,7 +805,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Image 3" descr="Picture"/>
+        <xdr:cNvPr id="7" name="Image 3" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -637,7 +842,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Image 4" descr="Picture"/>
+        <xdr:cNvPr id="8" name="Image 4" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -674,7 +879,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Image 5" descr="Picture"/>
+        <xdr:cNvPr id="9" name="Image 5" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -699,7 +904,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -710,13 +915,13 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>2370240</xdr:colOff>
+      <xdr:colOff>1084320</xdr:colOff>
       <xdr:row>4</xdr:row>
       <xdr:rowOff>2370240</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="Image 1" descr="Picture"/>
+        <xdr:cNvPr id="10" name="Image 1" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -726,7 +931,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="1236240" y="828720"/>
-          <a:ext cx="2332080" cy="2332080"/>
+          <a:ext cx="1046160" cy="2332080"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -747,13 +952,13 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>2370240</xdr:colOff>
+      <xdr:colOff>1084320</xdr:colOff>
       <xdr:row>5</xdr:row>
       <xdr:rowOff>2370240</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="6" name="Image 2" descr="Picture"/>
+        <xdr:cNvPr id="11" name="Image 2" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -763,7 +968,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="1236240" y="3238560"/>
-          <a:ext cx="2332080" cy="2332080"/>
+          <a:ext cx="1046160" cy="2332080"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -786,11 +991,11 @@
       <xdr:col>2</xdr:col>
       <xdr:colOff>2370240</xdr:colOff>
       <xdr:row>6</xdr:row>
-      <xdr:rowOff>2370240</xdr:rowOff>
+      <xdr:rowOff>1084320</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="7" name="Image 3" descr="Picture"/>
+        <xdr:cNvPr id="12" name="Image 3" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -800,7 +1005,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="1236240" y="5648400"/>
-          <a:ext cx="2332080" cy="2332080"/>
+          <a:ext cx="2332080" cy="1046160"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -821,13 +1026,13 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>2370240</xdr:colOff>
+      <xdr:colOff>1084320</xdr:colOff>
       <xdr:row>7</xdr:row>
       <xdr:rowOff>2370240</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="8" name="Image 4" descr="Picture"/>
+        <xdr:cNvPr id="13" name="Image 4" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -837,7 +1042,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="1236240" y="8058240"/>
-          <a:ext cx="2332080" cy="2332080"/>
+          <a:ext cx="1046160" cy="2332080"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -864,7 +1069,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="9" name="Image 5" descr="Picture"/>
+        <xdr:cNvPr id="14" name="Image 5" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -889,7 +1094,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -900,13 +1105,13 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>1084680</xdr:colOff>
+      <xdr:colOff>2370600</xdr:colOff>
       <xdr:row>4</xdr:row>
       <xdr:rowOff>2370600</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="10" name="Image 1" descr="Picture"/>
+        <xdr:cNvPr id="15" name="Image 1" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -916,7 +1121,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="1236240" y="828720"/>
-          <a:ext cx="1046520" cy="2332440"/>
+          <a:ext cx="2332440" cy="2332440"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -937,13 +1142,13 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>1084680</xdr:colOff>
+      <xdr:colOff>2370600</xdr:colOff>
       <xdr:row>5</xdr:row>
       <xdr:rowOff>2370600</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="11" name="Image 2" descr="Picture"/>
+        <xdr:cNvPr id="16" name="Image 2" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -953,7 +1158,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="1236240" y="3238560"/>
-          <a:ext cx="1046520" cy="2332440"/>
+          <a:ext cx="2332440" cy="2332440"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -976,11 +1181,11 @@
       <xdr:col>2</xdr:col>
       <xdr:colOff>2370600</xdr:colOff>
       <xdr:row>6</xdr:row>
-      <xdr:rowOff>1084680</xdr:rowOff>
+      <xdr:rowOff>2370600</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="12" name="Image 3" descr="Picture"/>
+        <xdr:cNvPr id="17" name="Image 3" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -990,7 +1195,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="1236240" y="5648400"/>
-          <a:ext cx="2332440" cy="1046520"/>
+          <a:ext cx="2332440" cy="2332440"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1011,13 +1216,13 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>1084680</xdr:colOff>
+      <xdr:colOff>2370600</xdr:colOff>
       <xdr:row>7</xdr:row>
       <xdr:rowOff>2370600</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="13" name="Image 4" descr="Picture"/>
+        <xdr:cNvPr id="18" name="Image 4" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -1027,7 +1232,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="1236240" y="8058240"/>
-          <a:ext cx="1046520" cy="2332440"/>
+          <a:ext cx="2332440" cy="2332440"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1054,7 +1259,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="14" name="Image 5" descr="Picture"/>
+        <xdr:cNvPr id="19" name="Image 5" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -1065,196 +1270,6 @@
         <a:xfrm>
           <a:off x="1236240" y="10468080"/>
           <a:ext cx="2332440" cy="2332440"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="0">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>38160</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>38160</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>2370960</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>2370960</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="15" name="Image 1" descr="Picture"/>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId1"/>
-        <a:stretch/>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="1236240" y="828720"/>
-          <a:ext cx="2332800" cy="2332800"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="0">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>38160</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>38160</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>2370960</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>2370960</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="16" name="Image 2" descr="Picture"/>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId2"/>
-        <a:stretch/>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="1236240" y="3238560"/>
-          <a:ext cx="2332800" cy="2332800"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="0">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>38160</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>38160</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>2370960</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>2370960</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="17" name="Image 3" descr="Picture"/>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId3"/>
-        <a:stretch/>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="1236240" y="5648400"/>
-          <a:ext cx="2332800" cy="2332800"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="0">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>38160</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>38160</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>2370960</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>2370960</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="18" name="Image 4" descr="Picture"/>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId4"/>
-        <a:stretch/>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="1236240" y="8058240"/>
-          <a:ext cx="2332800" cy="2332800"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="0">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>38160</xdr:colOff>
-      <xdr:row>8</xdr:row>
-      <xdr:rowOff>38160</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>2370960</xdr:colOff>
-      <xdr:row>8</xdr:row>
-      <xdr:rowOff>2370960</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="19" name="Image 5" descr="Picture"/>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId5"/>
-        <a:stretch/>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="1236240" y="10468080"/>
-          <a:ext cx="2332800" cy="2332800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1280,9 +1295,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>2371320</xdr:colOff>
+      <xdr:colOff>2370960</xdr:colOff>
       <xdr:row>4</xdr:row>
-      <xdr:rowOff>2371320</xdr:rowOff>
+      <xdr:rowOff>2370960</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1296,7 +1311,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="2223360" y="828720"/>
-          <a:ext cx="2333160" cy="2333160"/>
+          <a:ext cx="2332800" cy="2332800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1317,9 +1332,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>2371320</xdr:colOff>
+      <xdr:colOff>2370960</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>2371320</xdr:rowOff>
+      <xdr:rowOff>2370960</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1333,6 +1348,196 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="2223360" y="3238560"/>
+          <a:ext cx="2332800" cy="2332800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>38160</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>38160</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>2371320</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>2371320</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="22" name="Image 1" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1236240" y="828720"/>
+          <a:ext cx="2333160" cy="2333160"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>38160</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>38160</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>2371320</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>2371320</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="23" name="Image 2" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId2"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1236240" y="3238560"/>
+          <a:ext cx="2333160" cy="2333160"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>38160</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>38160</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>2371320</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>2371320</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="24" name="Image 3" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId3"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1236240" y="5648400"/>
+          <a:ext cx="2333160" cy="2333160"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>38160</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>38160</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>2371320</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>2371320</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="25" name="Image 4" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId4"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1236240" y="8058240"/>
+          <a:ext cx="2333160" cy="2333160"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>38160</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>38160</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>2371320</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>2371320</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="26" name="Image 5" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId5"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1236240" y="10468080"/>
           <a:ext cx="2333160" cy="2333160"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1678,7 +1883,7 @@
       </c>
       <c r="B13" s="6" t="n">
         <f aca="false">COUNTA('VZT 5.1'!D5:D24)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="C13" s="7" t="str">
         <f aca="false">IF(COUNT('VZT 5.1'!B5:B24)=0,"",MAX('VZT 5.1'!B5:B24))</f>
@@ -1720,7 +1925,7 @@
       </c>
       <c r="B16" s="9" t="n">
         <f aca="false">SUM(B5:B15)</f>
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="C16" s="10"/>
       <c r="D16" s="10"/>
@@ -1792,7 +1997,9 @@
       </c>
       <c r="B5" s="13"/>
       <c r="C5" s="14"/>
-      <c r="D5" s="15"/>
+      <c r="D5" s="15" t="s">
+        <v>55</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="189.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="12" t="n">
@@ -1800,7 +2007,9 @@
       </c>
       <c r="B6" s="13"/>
       <c r="C6" s="14"/>
-      <c r="D6" s="15"/>
+      <c r="D6" s="15" t="s">
+        <v>56</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="189.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="12" t="n">
@@ -1808,7 +2017,9 @@
       </c>
       <c r="B7" s="13"/>
       <c r="C7" s="14"/>
-      <c r="D7" s="15"/>
+      <c r="D7" s="15" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="189.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="12" t="n">
@@ -1816,7 +2027,9 @@
       </c>
       <c r="B8" s="13"/>
       <c r="C8" s="14"/>
-      <c r="D8" s="15"/>
+      <c r="D8" s="15" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="189.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="12" t="n">
@@ -1824,7 +2037,9 @@
       </c>
       <c r="B9" s="13"/>
       <c r="C9" s="14"/>
-      <c r="D9" s="15"/>
+      <c r="D9" s="15" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="189.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="12" t="n">
@@ -1954,6 +2169,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1972,7 +2188,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2180,7 +2396,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Add VZT 10.1 photos with draft captions
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DkBvnLE3negxmtmFidQ4SP
</commit_message>
<xml_diff>
--- a/vystupy/Fotodokumentace_VZT_prehled.xlsx
+++ b/vystupy/Fotodokumentace_VZT_prehled.xlsx
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="67">
   <si>
     <t xml:space="preserve">Přehled fotodokumentace úprav VZT – Mondelez Werk 2</t>
   </si>
@@ -227,6 +227,21 @@
   </si>
   <si>
     <t xml:space="preserve">Fotodokumentace provedených úprav – VZT 10.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Detail prostupu kabelu do stávající jednotky – bílý kabel s průchodkou, ohebná chránička, poškozená a odlepená hliníková izolace, stopy rzi.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stávající jednotka na střeše (původní provedení) – kabely v ohebných chráničkách, na střeše dvě nová potrubní tělesa odložená vedle.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stávající jednotka – klapka s pohonem Belimo, kabelová krabice na boku, kabely v chráničkách.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pohled na jednotku a odložené nové potrubní těleso (otevřený ocelový box) na střeše.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Celkový pohled na stávající jednotku s přilehlým potrubím a nově dodanými díly na střeše.</t>
   </si>
   <si>
     <t xml:space="preserve">Fotodokumentace provedených úprav – Odpad</t>
@@ -535,13 +550,203 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
+      <xdr:colOff>2369160</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>2369160</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="0" name="Image 1" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1236240" y="828720"/>
+          <a:ext cx="2331000" cy="2331000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>38160</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>38160</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>2369160</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>2369160</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="Image 2" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId2"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1236240" y="3238560"/>
+          <a:ext cx="2331000" cy="2331000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>38160</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>38160</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>2369160</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>2369160</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Image 3" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId3"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1236240" y="5648400"/>
+          <a:ext cx="2331000" cy="2331000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>38160</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>38160</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>2369160</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>2369160</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Image 4" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId4"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1236240" y="8058240"/>
+          <a:ext cx="2331000" cy="2331000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>38160</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>38160</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>2369160</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>2369160</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Image 5" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId5"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1236240" y="10468080"/>
+          <a:ext cx="2331000" cy="2331000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>38160</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>38160</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
       <xdr:colOff>2369520</xdr:colOff>
       <xdr:row>4</xdr:row>
       <xdr:rowOff>2369520</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="Image 1" descr="Picture"/>
+        <xdr:cNvPr id="5" name="Image 1" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -578,7 +783,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="Image 2" descr="Picture"/>
+        <xdr:cNvPr id="6" name="Image 2" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -615,7 +820,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Image 3" descr="Picture"/>
+        <xdr:cNvPr id="7" name="Image 3" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -652,7 +857,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Image 4" descr="Picture"/>
+        <xdr:cNvPr id="8" name="Image 4" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -689,7 +894,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Image 5" descr="Picture"/>
+        <xdr:cNvPr id="9" name="Image 5" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -714,7 +919,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -725,13 +930,13 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>2369880</xdr:colOff>
+      <xdr:colOff>1083960</xdr:colOff>
       <xdr:row>4</xdr:row>
       <xdr:rowOff>2369880</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="Image 1" descr="Picture"/>
+        <xdr:cNvPr id="10" name="Image 1" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -741,7 +946,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="1236240" y="828720"/>
-          <a:ext cx="2331720" cy="2331720"/>
+          <a:ext cx="1045800" cy="2331720"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -762,13 +967,13 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>2369880</xdr:colOff>
+      <xdr:colOff>1083960</xdr:colOff>
       <xdr:row>5</xdr:row>
       <xdr:rowOff>2369880</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="6" name="Image 2" descr="Picture"/>
+        <xdr:cNvPr id="11" name="Image 2" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -778,7 +983,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="1236240" y="3238560"/>
-          <a:ext cx="2331720" cy="2331720"/>
+          <a:ext cx="1045800" cy="2331720"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -801,11 +1006,11 @@
       <xdr:col>2</xdr:col>
       <xdr:colOff>2369880</xdr:colOff>
       <xdr:row>6</xdr:row>
-      <xdr:rowOff>2369880</xdr:rowOff>
+      <xdr:rowOff>1083960</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="7" name="Image 3" descr="Picture"/>
+        <xdr:cNvPr id="12" name="Image 3" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -815,7 +1020,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="1236240" y="5648400"/>
-          <a:ext cx="2331720" cy="2331720"/>
+          <a:ext cx="2331720" cy="1045800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -836,13 +1041,13 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>2369880</xdr:colOff>
+      <xdr:colOff>1083960</xdr:colOff>
       <xdr:row>7</xdr:row>
       <xdr:rowOff>2369880</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="8" name="Image 4" descr="Picture"/>
+        <xdr:cNvPr id="13" name="Image 4" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -852,7 +1057,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="1236240" y="8058240"/>
-          <a:ext cx="2331720" cy="2331720"/>
+          <a:ext cx="1045800" cy="2331720"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -879,7 +1084,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="9" name="Image 5" descr="Picture"/>
+        <xdr:cNvPr id="14" name="Image 5" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -904,7 +1109,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -915,13 +1120,13 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>1084320</xdr:colOff>
+      <xdr:colOff>2370240</xdr:colOff>
       <xdr:row>4</xdr:row>
       <xdr:rowOff>2370240</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="10" name="Image 1" descr="Picture"/>
+        <xdr:cNvPr id="15" name="Image 1" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -931,7 +1136,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="1236240" y="828720"/>
-          <a:ext cx="1046160" cy="2332080"/>
+          <a:ext cx="2332080" cy="2332080"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -952,13 +1157,13 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>1084320</xdr:colOff>
+      <xdr:colOff>2370240</xdr:colOff>
       <xdr:row>5</xdr:row>
       <xdr:rowOff>2370240</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="11" name="Image 2" descr="Picture"/>
+        <xdr:cNvPr id="16" name="Image 2" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -968,7 +1173,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="1236240" y="3238560"/>
-          <a:ext cx="1046160" cy="2332080"/>
+          <a:ext cx="2332080" cy="2332080"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -991,11 +1196,11 @@
       <xdr:col>2</xdr:col>
       <xdr:colOff>2370240</xdr:colOff>
       <xdr:row>6</xdr:row>
-      <xdr:rowOff>1084320</xdr:rowOff>
+      <xdr:rowOff>2370240</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="12" name="Image 3" descr="Picture"/>
+        <xdr:cNvPr id="17" name="Image 3" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -1005,7 +1210,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="1236240" y="5648400"/>
-          <a:ext cx="2332080" cy="1046160"/>
+          <a:ext cx="2332080" cy="2332080"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1026,13 +1231,13 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>1084320</xdr:colOff>
+      <xdr:colOff>2370240</xdr:colOff>
       <xdr:row>7</xdr:row>
       <xdr:rowOff>2370240</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="13" name="Image 4" descr="Picture"/>
+        <xdr:cNvPr id="18" name="Image 4" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -1042,7 +1247,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="1236240" y="8058240"/>
-          <a:ext cx="1046160" cy="2332080"/>
+          <a:ext cx="2332080" cy="2332080"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1069,7 +1274,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="14" name="Image 5" descr="Picture"/>
+        <xdr:cNvPr id="19" name="Image 5" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -1080,196 +1285,6 @@
         <a:xfrm>
           <a:off x="1236240" y="10468080"/>
           <a:ext cx="2332080" cy="2332080"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="0">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>38160</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>38160</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>2370600</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>2370600</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="15" name="Image 1" descr="Picture"/>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId1"/>
-        <a:stretch/>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="1236240" y="828720"/>
-          <a:ext cx="2332440" cy="2332440"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="0">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>38160</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>38160</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>2370600</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>2370600</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="16" name="Image 2" descr="Picture"/>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId2"/>
-        <a:stretch/>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="1236240" y="3238560"/>
-          <a:ext cx="2332440" cy="2332440"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="0">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>38160</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>38160</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>2370600</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>2370600</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="17" name="Image 3" descr="Picture"/>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId3"/>
-        <a:stretch/>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="1236240" y="5648400"/>
-          <a:ext cx="2332440" cy="2332440"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="0">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>38160</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>38160</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>2370600</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>2370600</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="18" name="Image 4" descr="Picture"/>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId4"/>
-        <a:stretch/>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="1236240" y="8058240"/>
-          <a:ext cx="2332440" cy="2332440"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="0">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>38160</xdr:colOff>
-      <xdr:row>8</xdr:row>
-      <xdr:rowOff>38160</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>2370600</xdr:colOff>
-      <xdr:row>8</xdr:row>
-      <xdr:rowOff>2370600</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="19" name="Image 5" descr="Picture"/>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId5"/>
-        <a:stretch/>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="1236240" y="10468080"/>
-          <a:ext cx="2332440" cy="2332440"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1295,9 +1310,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>2370960</xdr:colOff>
+      <xdr:colOff>2370600</xdr:colOff>
       <xdr:row>4</xdr:row>
-      <xdr:rowOff>2370960</xdr:rowOff>
+      <xdr:rowOff>2370600</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1311,7 +1326,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="2223360" y="828720"/>
-          <a:ext cx="2332800" cy="2332800"/>
+          <a:ext cx="2332440" cy="2332440"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1332,9 +1347,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>2370960</xdr:colOff>
+      <xdr:colOff>2370600</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>2370960</xdr:rowOff>
+      <xdr:rowOff>2370600</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1348,7 +1363,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="2223360" y="3238560"/>
-          <a:ext cx="2332800" cy="2332800"/>
+          <a:ext cx="2332440" cy="2332440"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1374,13 +1389,203 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
+      <xdr:colOff>2370960</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>2370960</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="22" name="Image 1" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1236240" y="828720"/>
+          <a:ext cx="2332800" cy="2332800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>38160</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>38160</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>2370960</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>2370960</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="23" name="Image 2" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId2"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1236240" y="3238560"/>
+          <a:ext cx="2332800" cy="2332800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>38160</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>38160</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>2370960</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>2370960</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="24" name="Image 3" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId3"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1236240" y="5648400"/>
+          <a:ext cx="2332800" cy="2332800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>38160</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>38160</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>2370960</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>2370960</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="25" name="Image 4" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId4"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1236240" y="8058240"/>
+          <a:ext cx="2332800" cy="2332800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>38160</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>38160</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>2370960</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>2370960</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="26" name="Image 5" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId5"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1236240" y="10468080"/>
+          <a:ext cx="2332800" cy="2332800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>38160</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>38160</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
       <xdr:colOff>2371320</xdr:colOff>
       <xdr:row>4</xdr:row>
       <xdr:rowOff>2371320</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="22" name="Image 1" descr="Picture"/>
+        <xdr:cNvPr id="27" name="Image 1" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -1417,7 +1622,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="23" name="Image 2" descr="Picture"/>
+        <xdr:cNvPr id="28" name="Image 2" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -1454,7 +1659,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="24" name="Image 3" descr="Picture"/>
+        <xdr:cNvPr id="29" name="Image 3" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -1491,7 +1696,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="25" name="Image 4" descr="Picture"/>
+        <xdr:cNvPr id="30" name="Image 4" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -1528,7 +1733,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="26" name="Image 5" descr="Picture"/>
+        <xdr:cNvPr id="31" name="Image 5" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -1897,7 +2102,7 @@
       </c>
       <c r="B14" s="6" t="n">
         <f aca="false">COUNTA('VZT 10.1'!D5:D24)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="C14" s="7" t="str">
         <f aca="false">IF(COUNT('VZT 10.1'!B5:B24)=0,"",MAX('VZT 10.1'!B5:B24))</f>
@@ -1925,7 +2130,7 @@
       </c>
       <c r="B16" s="9" t="n">
         <f aca="false">SUM(B5:B15)</f>
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="C16" s="10"/>
       <c r="D16" s="10"/>
@@ -2216,7 +2421,9 @@
       </c>
       <c r="B5" s="13"/>
       <c r="C5" s="14"/>
-      <c r="D5" s="15"/>
+      <c r="D5" s="15" t="s">
+        <v>61</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="189.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="12" t="n">
@@ -2224,7 +2431,9 @@
       </c>
       <c r="B6" s="13"/>
       <c r="C6" s="14"/>
-      <c r="D6" s="15"/>
+      <c r="D6" s="15" t="s">
+        <v>62</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="189.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="12" t="n">
@@ -2232,7 +2441,9 @@
       </c>
       <c r="B7" s="13"/>
       <c r="C7" s="14"/>
-      <c r="D7" s="15"/>
+      <c r="D7" s="15" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="189.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="12" t="n">
@@ -2240,7 +2451,9 @@
       </c>
       <c r="B8" s="13"/>
       <c r="C8" s="14"/>
-      <c r="D8" s="15"/>
+      <c r="D8" s="15" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="189.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="12" t="n">
@@ -2248,7 +2461,9 @@
       </c>
       <c r="B9" s="13"/>
       <c r="C9" s="14"/>
-      <c r="D9" s="15"/>
+      <c r="D9" s="15" t="s">
+        <v>65</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="189.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="12" t="n">
@@ -2378,6 +2593,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2396,7 +2612,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>